<commit_message>
modify database and report
</commit_message>
<xml_diff>
--- a/database.xlsx
+++ b/database.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/janice/Documents/hubble-constant-measurement-methods/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0FF1BD69-5E94-8145-A0CE-92E73629C640}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F2CB1834-5D3F-AD42-8516-27AF53809E51}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="660" windowWidth="29400" windowHeight="16940" xr2:uid="{A695B320-A17B-DD4C-82CF-5075F2BCF041}"/>
   </bookViews>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="478" uniqueCount="323">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="480" uniqueCount="323">
   <si>
     <t>Method</t>
   </si>
@@ -219,24 +219,10 @@
     <t>luminosity distance, detector-frame chirp mass</t>
   </si>
   <si>
-    <t>There are identifiable features in the source-frame mass spectrum of black holes (e.g. the pair-instability mass gap), which allow the redshift to be inferred by comparing the detector-frame and assumed source-frame masses.</t>
-  </si>
-  <si>
-    <t>&lt;0.8</t>
-  </si>
-  <si>
     <t>compact object merger (BNS, NSBH)</t>
   </si>
   <si>
     <t>km-scale laser-interferometer GW detector network with kHz high-frequency sensitivity (LIGO Hanford + Livingston, Virgo, KAGRA)</t>
-  </si>
-  <si>
-    <t>Neutron stars experience tidal deformation during inspiral.
-Tidal deformation parameters can be inferred from the GW phase evolution; combined with an assumed equation of state, this yields the source-frame mass.
-Comparing the detector-frame and source-frame mass then determines the redshift.</t>
-  </si>
-  <si>
-    <t>&lt;4</t>
   </si>
   <si>
     <t>GW phase evolution</t>
@@ -751,14 +737,6 @@
   </si>
   <si>
     <t>wide-aperture low-dispersion optical spectrograph for spectrophotometry (e.g. OAN-SPM 2.1 m/Boller &amp; Chivens spectrograph)</t>
-  </si>
-  <si>
-    <t>Distance:
-The HII galaxies and giant HII regions are empirically found to follow a common relation between H$\beta$ luminosity and the velocity dispersion of the ionised gas.
-The relation's zero point is calibrated using giant HII regions in nearby galaxies with independently measured distances.
-The measured velocity dispersion predicts the intrinsic H$\beta$ luminosity, which, when compared with the spectrophotometrically measured H$\beta$ flux, yields the luminosity distance.
-Velocity:
-Spectroscopic redshifts of Hubble-flow H II galaxies.</t>
   </si>
   <si>
     <t>0.01-7.5</t>
@@ -916,9 +894,6 @@
     <t>wide-field optical/near-IR imaging facilities with multi-wavelength follow-up</t>
   </si>
   <si>
-    <t>km-scale laser-interferometer GW detector network (LIGO, Virgo, KAGRA)</t>
-  </si>
-  <si>
     <t>[{"text": "Abbott et al. 2017","url": "https://doi.org/10.1038/nature24471"}]</t>
   </si>
   <si>
@@ -932,12 +907,6 @@
   </si>
   <si>
     <t>radio interferometric array (e.g. OVRO, BIMA)</t>
-  </si>
-  <si>
-    <t>Gamma-ray photons from blazars pair-produce with EBL photons while propagating over cosmological distances, attenuating the observed spectrum in an energy- and redshift-dependent way.
-Comparing observed blazar spectra against an assumed intrinsic spectral shape yields the observed optical depth.
-The same optical depth can also be predicted theoretically, by combining EBL density and path length to that redshift, which depends on $H_0$.
-Fitting the predicted and observed optical depth constrains $H_0$.</t>
   </si>
   <si>
     <t>temperature</t>
@@ -1085,9 +1054,6 @@
   </si>
   <si>
     <t>Physical Quantity: physical quantity inferred or measured from the observational data</t>
-  </si>
-  <si>
-    <t>Redshift Range: redshift range directly used in published measurements or inferences of $H_0$</t>
   </si>
   <si>
     <t>Physical Quantity</t>
@@ -1256,6 +1222,43 @@
   </si>
   <si>
     <t>$\leq 3.1$</t>
+  </si>
+  <si>
+    <t>Distance:
+The GW waveform's amplitude and phase jointly provide the chirp mass and luminosity distance.
+Redshift:
+There are identifiable features in the source-frame mass spectrum of black holes (e.g. the pair-instability mass gap), which allow the redshift to be inferred by comparing the detector-frame and assumed source-frame masses.</t>
+  </si>
+  <si>
+    <t>Redshift Range: redshift range directly used in published $H_0$ measurements or inferences when available; otherwise, the forecast redshift range for methods not yet applied to $H_0$ measurements</t>
+  </si>
+  <si>
+    <t>$z \lesssim 1$</t>
+  </si>
+  <si>
+    <t>[{"text": "Magaña Hernandez &amp; Palmese 2025","url": "https://arxiv.org/abs/2509.03607"}]</t>
+  </si>
+  <si>
+    <t>km-scale laser-interferometer GW detector network (e.g. LIGO, Virgo, KAGRA)</t>
+  </si>
+  <si>
+    <t>Distance:
+The GW waveform's amplitude and phase jointly provide the chirp mass and luminosity distance.
+Redshift:
+Neutron stars experience tidal deformation during inspiral.
+Tidal deformation parameters can be inferred from the GW phase evolution; combined with an assumed equation of state, this yields the source-frame mass.
+Comparing the detector-frame and source-frame mass then determines the redshift.</t>
+  </si>
+  <si>
+    <t>[{"text": "Chatterjee et al. 2021","url": "https://doi.org/10.1103/PhysRevD.104.083528"}]</t>
+  </si>
+  <si>
+    <t>Distance:
+The HII galaxies and giant HII regions are empirically found to follow a common relation between H$\beta$ luminosity and the velocity dispersion of the ionised gas.
+The relation's zero point is calibrated using giant HII regions in nearby galaxies with independently measured distances.
+The measured velocity dispersion predicts the intrinsic H$\beta$ luminosity, which, when compared with the spectrophotometrically measured H$\beta$ flux, yields the luminosity distance.
+Velocity:
+Spectroscopic redshifts of HII galaxies.</t>
   </si>
 </sst>
 </file>
@@ -1393,7 +1396,7 @@
       <name val="Aptos Narrow"/>
     </font>
   </fonts>
-  <fills count="5">
+  <fills count="3">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -1403,18 +1406,6 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="FFFFFF00"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="8" tint="0.79998168889431442"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="9" tint="0.79998168889431442"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -1431,7 +1422,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="47">
+  <cellXfs count="42">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -1478,9 +1469,6 @@
     <xf numFmtId="0" fontId="15" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="16" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="17" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
@@ -1496,15 +1484,13 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="16" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -1514,7 +1500,6 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
@@ -1527,9 +1512,6 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="16" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
@@ -1539,10 +1521,9 @@
     <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="17" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
@@ -1550,9 +1531,6 @@
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="11" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
@@ -1924,48 +1902,48 @@
         <v>1</v>
       </c>
       <c r="C1" s="1" t="s">
+        <v>259</v>
+      </c>
+      <c r="D1" s="1" t="s">
+        <v>260</v>
+      </c>
+      <c r="E1" s="1" t="s">
+        <v>204</v>
+      </c>
+      <c r="F1" s="1" t="s">
+        <v>272</v>
+      </c>
+      <c r="G1" s="1" t="s">
+        <v>295</v>
+      </c>
+      <c r="H1" s="1" t="s">
+        <v>238</v>
+      </c>
+      <c r="I1" s="1" t="s">
+        <v>273</v>
+      </c>
+      <c r="J1" s="1" t="s">
+        <v>252</v>
+      </c>
+      <c r="K1" s="1" t="s">
         <v>266</v>
       </c>
-      <c r="D1" s="1" t="s">
-        <v>267</v>
-      </c>
-      <c r="E1" s="1" t="s">
-        <v>209</v>
-      </c>
-      <c r="F1" s="1" t="s">
-        <v>280</v>
-      </c>
-      <c r="G1" s="1" t="s">
-        <v>303</v>
-      </c>
-      <c r="H1" s="1" t="s">
-        <v>245</v>
-      </c>
-      <c r="I1" s="1" t="s">
-        <v>281</v>
-      </c>
-      <c r="J1" s="1" t="s">
-        <v>259</v>
-      </c>
-      <c r="K1" s="1" t="s">
-        <v>273</v>
-      </c>
       <c r="L1" s="1" t="s">
-        <v>304</v>
+        <v>296</v>
       </c>
     </row>
     <row r="2" spans="1:14" ht="68" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A2" s="42" t="s">
-        <v>282</v>
-      </c>
-      <c r="B2" s="24" t="s">
-        <v>55</v>
-      </c>
-      <c r="C2" s="24" t="s">
+      <c r="A2" s="22" t="s">
+        <v>274</v>
+      </c>
+      <c r="B2" s="22" t="s">
+        <v>51</v>
+      </c>
+      <c r="C2" s="22" t="s">
         <v>3</v>
       </c>
       <c r="D2" s="3" t="s">
-        <v>296</v>
+        <v>288</v>
       </c>
       <c r="E2" s="4" t="s">
         <v>4</v>
@@ -1973,31 +1951,31 @@
       <c r="F2" s="2" t="s">
         <v>5</v>
       </c>
-      <c r="G2" s="27" t="s">
-        <v>285</v>
-      </c>
-      <c r="H2" s="24" t="s">
-        <v>246</v>
-      </c>
-      <c r="I2" s="24" t="s">
+      <c r="G2" s="26" t="s">
+        <v>277</v>
+      </c>
+      <c r="H2" s="22" t="s">
+        <v>239</v>
+      </c>
+      <c r="I2" s="22" t="s">
         <v>6</v>
       </c>
-      <c r="J2" s="24" t="s">
+      <c r="J2" s="22" t="s">
         <v>7</v>
       </c>
-      <c r="K2" s="24" t="s">
+      <c r="K2" s="22" t="s">
         <v>8</v>
       </c>
-      <c r="L2" s="24" t="s">
+      <c r="L2" s="22" t="s">
         <v>9</v>
       </c>
     </row>
     <row r="3" spans="1:14" ht="51" x14ac:dyDescent="0.2">
-      <c r="A3" s="42"/>
-      <c r="B3" s="24"/>
-      <c r="C3" s="24"/>
+      <c r="A3" s="22"/>
+      <c r="B3" s="22"/>
+      <c r="C3" s="22"/>
       <c r="D3" s="6" t="s">
-        <v>283</v>
+        <v>275</v>
       </c>
       <c r="E3" s="3" t="s">
         <v>10</v>
@@ -2005,20 +1983,20 @@
       <c r="F3" s="2" t="s">
         <v>11</v>
       </c>
-      <c r="G3" s="27"/>
-      <c r="H3" s="24"/>
-      <c r="I3" s="24"/>
-      <c r="J3" s="24"/>
-      <c r="K3" s="24"/>
-      <c r="L3" s="24"/>
-      <c r="N3" s="20"/>
+      <c r="G3" s="26"/>
+      <c r="H3" s="22"/>
+      <c r="I3" s="22"/>
+      <c r="J3" s="22"/>
+      <c r="K3" s="22"/>
+      <c r="L3" s="22"/>
+      <c r="N3" s="19"/>
     </row>
     <row r="4" spans="1:14" ht="51" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A4" s="42"/>
-      <c r="B4" s="24"/>
-      <c r="C4" s="24"/>
-      <c r="D4" s="31" t="s">
-        <v>284</v>
+      <c r="A4" s="22"/>
+      <c r="B4" s="22"/>
+      <c r="C4" s="22"/>
+      <c r="D4" s="29" t="s">
+        <v>276</v>
       </c>
       <c r="E4" s="7" t="s">
         <v>12</v>
@@ -2026,43 +2004,43 @@
       <c r="F4" s="2" t="s">
         <v>13</v>
       </c>
-      <c r="G4" s="27"/>
-      <c r="H4" s="24"/>
-      <c r="I4" s="24"/>
-      <c r="J4" s="24"/>
-      <c r="K4" s="24"/>
-      <c r="L4" s="24"/>
+      <c r="G4" s="26"/>
+      <c r="H4" s="22"/>
+      <c r="I4" s="22"/>
+      <c r="J4" s="22"/>
+      <c r="K4" s="22"/>
+      <c r="L4" s="22"/>
     </row>
     <row r="5" spans="1:14" ht="34" x14ac:dyDescent="0.2">
-      <c r="A5" s="42"/>
-      <c r="B5" s="24"/>
-      <c r="C5" s="24"/>
-      <c r="D5" s="31"/>
+      <c r="A5" s="22"/>
+      <c r="B5" s="22"/>
+      <c r="C5" s="22"/>
+      <c r="D5" s="29"/>
       <c r="E5" s="8" t="s">
         <v>14</v>
       </c>
       <c r="F5" s="2" t="s">
-        <v>311</v>
-      </c>
-      <c r="G5" s="27"/>
-      <c r="H5" s="24"/>
-      <c r="I5" s="24"/>
-      <c r="J5" s="24"/>
-      <c r="K5" s="24"/>
-      <c r="L5" s="24"/>
+        <v>303</v>
+      </c>
+      <c r="G5" s="26"/>
+      <c r="H5" s="22"/>
+      <c r="I5" s="22"/>
+      <c r="J5" s="22"/>
+      <c r="K5" s="22"/>
+      <c r="L5" s="22"/>
     </row>
     <row r="6" spans="1:14" ht="48" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A6" s="24" t="s">
+      <c r="A6" s="22" t="s">
         <v>15</v>
       </c>
-      <c r="B6" s="24" t="s">
-        <v>306</v>
-      </c>
-      <c r="C6" s="31" t="s">
+      <c r="B6" s="22" t="s">
+        <v>298</v>
+      </c>
+      <c r="C6" s="29" t="s">
         <v>16</v>
       </c>
-      <c r="D6" s="46" t="s">
-        <v>227</v>
+      <c r="D6" s="41" t="s">
+        <v>222</v>
       </c>
       <c r="E6" s="7" t="s">
         <v>17</v>
@@ -2070,51 +2048,51 @@
       <c r="F6" s="2" t="s">
         <v>18</v>
       </c>
-      <c r="G6" s="27" t="s">
+      <c r="G6" s="26" t="s">
         <v>19</v>
       </c>
-      <c r="H6" s="24" t="s">
-        <v>248</v>
-      </c>
-      <c r="I6" s="24" t="s">
+      <c r="H6" s="22" t="s">
+        <v>241</v>
+      </c>
+      <c r="I6" s="22" t="s">
         <v>20</v>
       </c>
-      <c r="J6" s="24" t="s">
+      <c r="J6" s="22" t="s">
         <v>7</v>
       </c>
-      <c r="K6" s="44" t="s">
+      <c r="K6" s="39" t="s">
         <v>8</v>
       </c>
-      <c r="L6" s="24" t="s">
+      <c r="L6" s="22" t="s">
         <v>21</v>
       </c>
     </row>
     <row r="7" spans="1:14" ht="53" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A7" s="24"/>
-      <c r="B7" s="24"/>
-      <c r="C7" s="24"/>
-      <c r="D7" s="24"/>
+      <c r="A7" s="22"/>
+      <c r="B7" s="22"/>
+      <c r="C7" s="22"/>
+      <c r="D7" s="22"/>
       <c r="E7" s="9" t="s">
         <v>22</v>
       </c>
       <c r="F7" s="2" t="s">
         <v>23</v>
       </c>
-      <c r="G7" s="32"/>
-      <c r="H7" s="24"/>
-      <c r="I7" s="28"/>
-      <c r="J7" s="24"/>
-      <c r="K7" s="45"/>
-      <c r="L7" s="28"/>
+      <c r="G7" s="30"/>
+      <c r="H7" s="22"/>
+      <c r="I7" s="23"/>
+      <c r="J7" s="22"/>
+      <c r="K7" s="40"/>
+      <c r="L7" s="23"/>
     </row>
     <row r="8" spans="1:14" ht="104" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A8" s="24"/>
-      <c r="B8" s="24"/>
+      <c r="A8" s="22"/>
+      <c r="B8" s="22"/>
       <c r="C8" s="11" t="s">
-        <v>226</v>
+        <v>221</v>
       </c>
       <c r="D8" s="7" t="s">
-        <v>225</v>
+        <v>220</v>
       </c>
       <c r="E8" s="7" t="s">
         <v>24</v>
@@ -2122,25 +2100,25 @@
       <c r="F8" s="2" t="s">
         <v>25</v>
       </c>
-      <c r="G8" s="32"/>
-      <c r="H8" s="24"/>
-      <c r="I8" s="28"/>
-      <c r="J8" s="24"/>
-      <c r="K8" s="45"/>
-      <c r="L8" s="28"/>
+      <c r="G8" s="30"/>
+      <c r="H8" s="22"/>
+      <c r="I8" s="23"/>
+      <c r="J8" s="22"/>
+      <c r="K8" s="40"/>
+      <c r="L8" s="23"/>
     </row>
     <row r="9" spans="1:14" ht="68" x14ac:dyDescent="0.2">
-      <c r="A9" s="42" t="s">
-        <v>286</v>
-      </c>
-      <c r="B9" s="24" t="s">
+      <c r="A9" s="22" t="s">
+        <v>278</v>
+      </c>
+      <c r="B9" s="22" t="s">
         <v>26</v>
       </c>
       <c r="C9" s="12" t="s">
         <v>27</v>
       </c>
       <c r="D9" s="4" t="s">
-        <v>229</v>
+        <v>319</v>
       </c>
       <c r="E9" s="13" t="s">
         <v>28</v>
@@ -2148,52 +2126,52 @@
       <c r="F9" s="2" t="s">
         <v>29</v>
       </c>
-      <c r="G9" s="27" t="s">
-        <v>231</v>
-      </c>
-      <c r="H9" s="24" t="s">
-        <v>246</v>
-      </c>
-      <c r="I9" s="24" t="s">
-        <v>320</v>
-      </c>
-      <c r="J9" s="24" t="s">
+      <c r="G9" s="26" t="s">
+        <v>225</v>
+      </c>
+      <c r="H9" s="22" t="s">
+        <v>239</v>
+      </c>
+      <c r="I9" s="22" t="s">
+        <v>312</v>
+      </c>
+      <c r="J9" s="22" t="s">
         <v>30</v>
       </c>
-      <c r="K9" s="24" t="s">
+      <c r="K9" s="22" t="s">
         <v>31</v>
       </c>
-      <c r="L9" s="24" t="s">
-        <v>230</v>
+      <c r="L9" s="22" t="s">
+        <v>224</v>
       </c>
     </row>
     <row r="10" spans="1:14" ht="98" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A10" s="42"/>
-      <c r="B10" s="24"/>
+      <c r="A10" s="22"/>
+      <c r="B10" s="22"/>
       <c r="C10" s="7" t="s">
         <v>32</v>
       </c>
       <c r="D10" s="6" t="s">
-        <v>228</v>
+        <v>223</v>
       </c>
       <c r="E10" s="3" t="s">
         <v>10</v>
       </c>
-      <c r="F10" s="24" t="s">
+      <c r="F10" s="22" t="s">
         <v>33</v>
       </c>
-      <c r="G10" s="32"/>
-      <c r="H10" s="24"/>
-      <c r="I10" s="28"/>
-      <c r="J10" s="24"/>
-      <c r="K10" s="28"/>
-      <c r="L10" s="28"/>
+      <c r="G10" s="30"/>
+      <c r="H10" s="22"/>
+      <c r="I10" s="23"/>
+      <c r="J10" s="22"/>
+      <c r="K10" s="23"/>
+      <c r="L10" s="23"/>
     </row>
     <row r="11" spans="1:14" ht="34" x14ac:dyDescent="0.2">
-      <c r="A11" s="42"/>
-      <c r="B11" s="24"/>
+      <c r="A11" s="22"/>
+      <c r="B11" s="22"/>
       <c r="C11" s="11" t="s">
-        <v>226</v>
+        <v>221</v>
       </c>
       <c r="D11" s="7" t="s">
         <v>34</v>
@@ -2201,24 +2179,24 @@
       <c r="E11" s="7" t="s">
         <v>12</v>
       </c>
-      <c r="F11" s="24"/>
-      <c r="G11" s="32"/>
-      <c r="H11" s="24"/>
-      <c r="I11" s="28"/>
-      <c r="J11" s="24"/>
-      <c r="K11" s="28"/>
-      <c r="L11" s="28"/>
+      <c r="F11" s="22"/>
+      <c r="G11" s="30"/>
+      <c r="H11" s="22"/>
+      <c r="I11" s="23"/>
+      <c r="J11" s="22"/>
+      <c r="K11" s="23"/>
+      <c r="L11" s="23"/>
     </row>
     <row r="12" spans="1:14" ht="85" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A12" s="42" t="s">
-        <v>287</v>
-      </c>
-      <c r="B12" s="24"/>
+      <c r="A12" s="22" t="s">
+        <v>279</v>
+      </c>
+      <c r="B12" s="22"/>
       <c r="C12" s="12" t="s">
         <v>35</v>
       </c>
       <c r="D12" s="4" t="s">
-        <v>229</v>
+        <v>319</v>
       </c>
       <c r="E12" s="13" t="s">
         <v>28</v>
@@ -2226,26 +2204,26 @@
       <c r="F12" s="2" t="s">
         <v>36</v>
       </c>
-      <c r="G12" s="27" t="s">
-        <v>294</v>
-      </c>
-      <c r="H12" s="24"/>
-      <c r="I12" s="24" t="s">
-        <v>290</v>
-      </c>
-      <c r="J12" s="24" t="s">
+      <c r="G12" s="26" t="s">
+        <v>286</v>
+      </c>
+      <c r="H12" s="22"/>
+      <c r="I12" s="22" t="s">
+        <v>282</v>
+      </c>
+      <c r="J12" s="22" t="s">
         <v>7</v>
       </c>
-      <c r="K12" s="24" t="s">
+      <c r="K12" s="22" t="s">
         <v>8</v>
       </c>
-      <c r="L12" s="24" t="s">
-        <v>291</v>
+      <c r="L12" s="22" t="s">
+        <v>283</v>
       </c>
     </row>
     <row r="13" spans="1:14" ht="69" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A13" s="42"/>
-      <c r="B13" s="24"/>
+      <c r="A13" s="22"/>
+      <c r="B13" s="22"/>
       <c r="C13" s="11" t="s">
         <v>37</v>
       </c>
@@ -2258,23 +2236,23 @@
       <c r="F13" s="2" t="s">
         <v>33</v>
       </c>
-      <c r="G13" s="32"/>
-      <c r="H13" s="24"/>
-      <c r="I13" s="28"/>
-      <c r="J13" s="24"/>
-      <c r="K13" s="28"/>
-      <c r="L13" s="28"/>
-    </row>
-    <row r="14" spans="1:14" ht="102" x14ac:dyDescent="0.2">
-      <c r="A14" s="22" t="s">
-        <v>288</v>
-      </c>
-      <c r="B14" s="24"/>
+      <c r="G13" s="30"/>
+      <c r="H13" s="22"/>
+      <c r="I13" s="23"/>
+      <c r="J13" s="22"/>
+      <c r="K13" s="23"/>
+      <c r="L13" s="23"/>
+    </row>
+    <row r="14" spans="1:14" ht="187" x14ac:dyDescent="0.2">
+      <c r="A14" s="2" t="s">
+        <v>280</v>
+      </c>
+      <c r="B14" s="22"/>
       <c r="C14" s="12" t="s">
         <v>35</v>
       </c>
       <c r="D14" s="4" t="s">
-        <v>229</v>
+        <v>319</v>
       </c>
       <c r="E14" s="13" t="s">
         <v>28</v>
@@ -2283,11 +2261,11 @@
         <v>39</v>
       </c>
       <c r="G14" s="5" t="s">
-        <v>40</v>
-      </c>
-      <c r="H14" s="24"/>
+        <v>315</v>
+      </c>
+      <c r="H14" s="22"/>
       <c r="I14" s="2" t="s">
-        <v>41</v>
+        <v>317</v>
       </c>
       <c r="J14" s="2" t="s">
         <v>7</v>
@@ -2295,18 +2273,20 @@
       <c r="K14" s="2" t="s">
         <v>8</v>
       </c>
-      <c r="L14" s="2"/>
+      <c r="L14" s="2" t="s">
+        <v>318</v>
+      </c>
     </row>
     <row r="15" spans="1:14" ht="71" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A15" s="37" t="s">
-        <v>289</v>
-      </c>
-      <c r="B15" s="24"/>
-      <c r="C15" s="43" t="s">
-        <v>42</v>
-      </c>
-      <c r="D15" s="41" t="s">
-        <v>43</v>
+      <c r="A15" s="22" t="s">
+        <v>281</v>
+      </c>
+      <c r="B15" s="22"/>
+      <c r="C15" s="38" t="s">
+        <v>40</v>
+      </c>
+      <c r="D15" s="37" t="s">
+        <v>41</v>
       </c>
       <c r="E15" s="13" t="s">
         <v>28</v>
@@ -2314,99 +2294,101 @@
       <c r="F15" s="2" t="s">
         <v>39</v>
       </c>
-      <c r="G15" s="27" t="s">
+      <c r="G15" s="26" t="s">
+        <v>320</v>
+      </c>
+      <c r="H15" s="22"/>
+      <c r="I15" s="22" t="s">
+        <v>317</v>
+      </c>
+      <c r="J15" s="22" t="s">
+        <v>7</v>
+      </c>
+      <c r="K15" s="22" t="s">
+        <v>8</v>
+      </c>
+      <c r="L15" s="22" t="s">
+        <v>321</v>
+      </c>
+    </row>
+    <row r="16" spans="1:14" ht="72" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A16" s="22"/>
+      <c r="B16" s="22"/>
+      <c r="C16" s="22"/>
+      <c r="D16" s="22"/>
+      <c r="E16" s="13" t="s">
+        <v>42</v>
+      </c>
+      <c r="F16" s="2" t="s">
+        <v>43</v>
+      </c>
+      <c r="G16" s="30"/>
+      <c r="H16" s="22"/>
+      <c r="I16" s="23"/>
+      <c r="J16" s="22"/>
+      <c r="K16" s="23"/>
+      <c r="L16" s="23"/>
+    </row>
+    <row r="17" spans="1:12" ht="63" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A17" s="22" t="s">
         <v>44</v>
       </c>
-      <c r="H15" s="24"/>
-      <c r="I15" s="24" t="s">
+      <c r="B17" s="22" t="s">
+        <v>298</v>
+      </c>
+      <c r="C17" s="33" t="s">
         <v>45</v>
       </c>
-      <c r="J15" s="24" t="s">
+      <c r="D17" s="3" t="s">
+        <v>313</v>
+      </c>
+      <c r="E17" s="29" t="s">
+        <v>12</v>
+      </c>
+      <c r="F17" s="22" t="s">
+        <v>46</v>
+      </c>
+      <c r="G17" s="26" t="s">
+        <v>315</v>
+      </c>
+      <c r="H17" s="22" t="s">
+        <v>241</v>
+      </c>
+      <c r="I17" s="22" t="s">
+        <v>314</v>
+      </c>
+      <c r="J17" s="22" t="s">
         <v>7</v>
       </c>
-      <c r="K15" s="24" t="s">
+      <c r="K17" s="22" t="s">
         <v>8</v>
       </c>
-      <c r="L15" s="24"/>
-    </row>
-    <row r="16" spans="1:14" ht="72" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A16" s="37"/>
-      <c r="B16" s="24"/>
-      <c r="C16" s="24"/>
-      <c r="D16" s="24"/>
-      <c r="E16" s="13" t="s">
-        <v>46</v>
-      </c>
-      <c r="F16" s="2" t="s">
+      <c r="L17" s="22" t="s">
         <v>47</v>
       </c>
-      <c r="G16" s="32"/>
-      <c r="H16" s="24"/>
-      <c r="I16" s="28"/>
-      <c r="J16" s="24"/>
-      <c r="K16" s="28"/>
-      <c r="L16" s="28"/>
-    </row>
-    <row r="17" spans="1:12" ht="63" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A17" s="37" t="s">
+    </row>
+    <row r="18" spans="1:12" ht="119" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A18" s="22"/>
+      <c r="B18" s="22"/>
+      <c r="C18" s="22"/>
+      <c r="D18" s="3" t="s">
         <v>48</v>
       </c>
-      <c r="B17" s="24" t="s">
-        <v>306</v>
-      </c>
-      <c r="C17" s="36" t="s">
+      <c r="E18" s="22"/>
+      <c r="F18" s="22"/>
+      <c r="G18" s="30"/>
+      <c r="H18" s="22"/>
+      <c r="I18" s="23"/>
+      <c r="J18" s="22"/>
+      <c r="K18" s="23"/>
+      <c r="L18" s="23"/>
+    </row>
+    <row r="19" spans="1:12" ht="51" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A19" s="22"/>
+      <c r="B19" s="22"/>
+      <c r="C19" s="22"/>
+      <c r="D19" s="7" t="s">
         <v>49</v>
-      </c>
-      <c r="D17" s="3" t="s">
-        <v>321</v>
-      </c>
-      <c r="E17" s="31" t="s">
-        <v>12</v>
-      </c>
-      <c r="F17" s="24" t="s">
-        <v>50</v>
-      </c>
-      <c r="G17" s="27" t="s">
-        <v>234</v>
-      </c>
-      <c r="H17" s="24" t="s">
-        <v>248</v>
-      </c>
-      <c r="I17" s="24" t="s">
-        <v>322</v>
-      </c>
-      <c r="J17" s="24" t="s">
-        <v>7</v>
-      </c>
-      <c r="K17" s="24" t="s">
-        <v>8</v>
-      </c>
-      <c r="L17" s="24" t="s">
-        <v>51</v>
-      </c>
-    </row>
-    <row r="18" spans="1:12" ht="119" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A18" s="37"/>
-      <c r="B18" s="24"/>
-      <c r="C18" s="24"/>
-      <c r="D18" s="3" t="s">
-        <v>52</v>
-      </c>
-      <c r="E18" s="24"/>
-      <c r="F18" s="24"/>
-      <c r="G18" s="32"/>
-      <c r="H18" s="24"/>
-      <c r="I18" s="28"/>
-      <c r="J18" s="24"/>
-      <c r="K18" s="28"/>
-      <c r="L18" s="28"/>
-    </row>
-    <row r="19" spans="1:12" ht="51" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A19" s="37"/>
-      <c r="B19" s="24"/>
-      <c r="C19" s="24"/>
-      <c r="D19" s="7" t="s">
-        <v>53</v>
       </c>
       <c r="E19" s="7" t="s">
         <v>12</v>
@@ -2414,95 +2396,95 @@
       <c r="F19" s="2" t="s">
         <v>33</v>
       </c>
-      <c r="G19" s="32"/>
-      <c r="H19" s="24"/>
-      <c r="I19" s="28"/>
-      <c r="J19" s="24"/>
-      <c r="K19" s="28"/>
-      <c r="L19" s="28"/>
+      <c r="G19" s="30"/>
+      <c r="H19" s="22"/>
+      <c r="I19" s="23"/>
+      <c r="J19" s="22"/>
+      <c r="K19" s="23"/>
+      <c r="L19" s="23"/>
     </row>
     <row r="20" spans="1:12" ht="83" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A20" s="24" t="s">
-        <v>54</v>
-      </c>
-      <c r="B20" s="24" t="s">
-        <v>55</v>
-      </c>
-      <c r="C20" s="26" t="s">
-        <v>56</v>
+      <c r="A20" s="22" t="s">
+        <v>50</v>
+      </c>
+      <c r="B20" s="22" t="s">
+        <v>51</v>
+      </c>
+      <c r="C20" s="25" t="s">
+        <v>52</v>
       </c>
       <c r="D20" s="8" t="s">
-        <v>233</v>
+        <v>227</v>
       </c>
       <c r="E20" s="4" t="s">
         <v>4</v>
       </c>
       <c r="F20" s="2" t="s">
-        <v>57</v>
-      </c>
-      <c r="G20" s="27" t="s">
-        <v>236</v>
-      </c>
-      <c r="H20" s="24" t="s">
-        <v>246</v>
-      </c>
-      <c r="I20" s="24" t="s">
-        <v>238</v>
-      </c>
-      <c r="J20" s="24" t="s">
+        <v>53</v>
+      </c>
+      <c r="G20" s="26" t="s">
+        <v>229</v>
+      </c>
+      <c r="H20" s="22" t="s">
+        <v>239</v>
+      </c>
+      <c r="I20" s="22" t="s">
+        <v>231</v>
+      </c>
+      <c r="J20" s="22" t="s">
         <v>7</v>
       </c>
-      <c r="K20" s="24" t="s">
+      <c r="K20" s="22" t="s">
         <v>8</v>
       </c>
-      <c r="L20" s="24" t="s">
-        <v>58</v>
+      <c r="L20" s="22" t="s">
+        <v>54</v>
       </c>
     </row>
     <row r="21" spans="1:12" ht="41" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A21" s="24"/>
-      <c r="B21" s="24"/>
-      <c r="C21" s="26"/>
-      <c r="D21" s="31" t="s">
-        <v>59</v>
+      <c r="A21" s="22"/>
+      <c r="B21" s="22"/>
+      <c r="C21" s="25"/>
+      <c r="D21" s="29" t="s">
+        <v>55</v>
       </c>
       <c r="E21" s="4" t="s">
         <v>4</v>
       </c>
       <c r="F21" s="2" t="s">
-        <v>232</v>
-      </c>
-      <c r="G21" s="27"/>
-      <c r="H21" s="24"/>
-      <c r="I21" s="24"/>
-      <c r="J21" s="24"/>
-      <c r="K21" s="24"/>
-      <c r="L21" s="24"/>
+        <v>226</v>
+      </c>
+      <c r="G21" s="26"/>
+      <c r="H21" s="22"/>
+      <c r="I21" s="22"/>
+      <c r="J21" s="22"/>
+      <c r="K21" s="22"/>
+      <c r="L21" s="22"/>
     </row>
     <row r="22" spans="1:12" ht="54" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A22" s="24"/>
-      <c r="B22" s="24"/>
-      <c r="C22" s="26"/>
-      <c r="D22" s="31"/>
+      <c r="A22" s="22"/>
+      <c r="B22" s="22"/>
+      <c r="C22" s="25"/>
+      <c r="D22" s="29"/>
       <c r="E22" s="7" t="s">
         <v>12</v>
       </c>
       <c r="F22" s="2" t="s">
-        <v>235</v>
-      </c>
-      <c r="G22" s="27"/>
-      <c r="H22" s="24"/>
-      <c r="I22" s="24"/>
-      <c r="J22" s="24"/>
-      <c r="K22" s="24"/>
-      <c r="L22" s="24"/>
+        <v>228</v>
+      </c>
+      <c r="G22" s="26"/>
+      <c r="H22" s="22"/>
+      <c r="I22" s="22"/>
+      <c r="J22" s="22"/>
+      <c r="K22" s="22"/>
+      <c r="L22" s="22"/>
     </row>
     <row r="23" spans="1:12" ht="54" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A23" s="24"/>
-      <c r="B23" s="24"/>
-      <c r="C23" s="26"/>
+      <c r="A23" s="22"/>
+      <c r="B23" s="22"/>
+      <c r="C23" s="25"/>
       <c r="D23" s="7" t="s">
-        <v>53</v>
+        <v>49</v>
       </c>
       <c r="E23" s="7" t="s">
         <v>12</v>
@@ -2510,79 +2492,79 @@
       <c r="F23" s="2" t="s">
         <v>33</v>
       </c>
-      <c r="G23" s="27"/>
-      <c r="H23" s="24"/>
-      <c r="I23" s="24"/>
-      <c r="J23" s="24"/>
-      <c r="K23" s="24"/>
-      <c r="L23" s="24"/>
+      <c r="G23" s="26"/>
+      <c r="H23" s="22"/>
+      <c r="I23" s="22"/>
+      <c r="J23" s="22"/>
+      <c r="K23" s="22"/>
+      <c r="L23" s="22"/>
     </row>
     <row r="24" spans="1:12" ht="69" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A24" s="42" t="s">
-        <v>60</v>
-      </c>
-      <c r="B24" s="24" t="s">
-        <v>55</v>
-      </c>
-      <c r="C24" s="29" t="s">
-        <v>61</v>
+      <c r="A24" s="22" t="s">
+        <v>56</v>
+      </c>
+      <c r="B24" s="22" t="s">
+        <v>51</v>
+      </c>
+      <c r="C24" s="27" t="s">
+        <v>57</v>
       </c>
       <c r="D24" s="8" t="s">
-        <v>307</v>
+        <v>299</v>
       </c>
       <c r="E24" s="4" t="s">
         <v>4</v>
       </c>
       <c r="F24" s="2" t="s">
-        <v>62</v>
-      </c>
-      <c r="G24" s="27" t="s">
-        <v>309</v>
-      </c>
-      <c r="H24" s="24" t="s">
-        <v>246</v>
-      </c>
-      <c r="I24" s="24" t="s">
-        <v>63</v>
-      </c>
-      <c r="J24" s="24" t="s">
+        <v>58</v>
+      </c>
+      <c r="G24" s="26" t="s">
+        <v>301</v>
+      </c>
+      <c r="H24" s="22" t="s">
+        <v>239</v>
+      </c>
+      <c r="I24" s="22" t="s">
+        <v>59</v>
+      </c>
+      <c r="J24" s="22" t="s">
         <v>30</v>
       </c>
-      <c r="K24" s="24" t="s">
+      <c r="K24" s="22" t="s">
         <v>31</v>
       </c>
-      <c r="L24" s="24" t="s">
-        <v>310</v>
+      <c r="L24" s="22" t="s">
+        <v>302</v>
       </c>
     </row>
     <row r="25" spans="1:12" ht="84" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A25" s="42"/>
-      <c r="B25" s="24"/>
-      <c r="C25" s="29"/>
+      <c r="A25" s="22"/>
+      <c r="B25" s="22"/>
+      <c r="C25" s="27"/>
       <c r="D25" s="8" t="s">
-        <v>312</v>
+        <v>304</v>
       </c>
       <c r="E25" s="7" t="s">
         <v>12</v>
       </c>
       <c r="F25" s="2" t="s">
-        <v>64</v>
-      </c>
-      <c r="G25" s="27"/>
-      <c r="H25" s="24"/>
-      <c r="I25" s="24"/>
-      <c r="J25" s="24"/>
-      <c r="K25" s="24"/>
-      <c r="L25" s="24"/>
+        <v>60</v>
+      </c>
+      <c r="G25" s="26"/>
+      <c r="H25" s="22"/>
+      <c r="I25" s="22"/>
+      <c r="J25" s="22"/>
+      <c r="K25" s="22"/>
+      <c r="L25" s="22"/>
     </row>
     <row r="26" spans="1:12" ht="17" x14ac:dyDescent="0.2">
-      <c r="A26" s="42"/>
-      <c r="B26" s="24"/>
+      <c r="A26" s="22"/>
+      <c r="B26" s="22"/>
       <c r="C26" s="11" t="s">
-        <v>226</v>
+        <v>221</v>
       </c>
       <c r="D26" s="7" t="s">
-        <v>53</v>
+        <v>49</v>
       </c>
       <c r="E26" s="7" t="s">
         <v>12</v>
@@ -2590,98 +2572,98 @@
       <c r="F26" s="2" t="s">
         <v>33</v>
       </c>
-      <c r="G26" s="27"/>
-      <c r="H26" s="24"/>
-      <c r="I26" s="24"/>
-      <c r="J26" s="24"/>
-      <c r="K26" s="24"/>
-      <c r="L26" s="24"/>
+      <c r="G26" s="26"/>
+      <c r="H26" s="22"/>
+      <c r="I26" s="22"/>
+      <c r="J26" s="22"/>
+      <c r="K26" s="22"/>
+      <c r="L26" s="22"/>
     </row>
     <row r="27" spans="1:12" ht="62" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A27" s="24" t="s">
-        <v>65</v>
-      </c>
-      <c r="B27" s="24" t="s">
-        <v>55</v>
-      </c>
-      <c r="C27" s="31" t="s">
-        <v>66</v>
+      <c r="A27" s="22" t="s">
+        <v>61</v>
+      </c>
+      <c r="B27" s="22" t="s">
+        <v>51</v>
+      </c>
+      <c r="C27" s="29" t="s">
+        <v>62</v>
       </c>
       <c r="D27" s="6" t="s">
-        <v>67</v>
+        <v>63</v>
       </c>
       <c r="E27" s="3" t="s">
         <v>10</v>
       </c>
       <c r="F27" s="2" t="s">
-        <v>68</v>
-      </c>
-      <c r="G27" s="27" t="s">
-        <v>241</v>
-      </c>
-      <c r="H27" s="24" t="s">
-        <v>246</v>
-      </c>
-      <c r="I27" s="24" t="s">
-        <v>240</v>
-      </c>
-      <c r="J27" s="24" t="s">
+        <v>64</v>
+      </c>
+      <c r="G27" s="26" t="s">
+        <v>234</v>
+      </c>
+      <c r="H27" s="22" t="s">
+        <v>239</v>
+      </c>
+      <c r="I27" s="22" t="s">
+        <v>233</v>
+      </c>
+      <c r="J27" s="22" t="s">
         <v>30</v>
       </c>
-      <c r="K27" s="24" t="s">
+      <c r="K27" s="22" t="s">
         <v>8</v>
       </c>
-      <c r="L27" s="24" t="s">
-        <v>239</v>
+      <c r="L27" s="22" t="s">
+        <v>232</v>
       </c>
     </row>
     <row r="28" spans="1:12" ht="85" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A28" s="24"/>
-      <c r="B28" s="24"/>
-      <c r="C28" s="24"/>
+      <c r="A28" s="22"/>
+      <c r="B28" s="22"/>
+      <c r="C28" s="22"/>
       <c r="D28" s="7" t="s">
-        <v>69</v>
+        <v>65</v>
       </c>
       <c r="E28" s="7" t="s">
         <v>12</v>
       </c>
       <c r="F28" s="2" t="s">
-        <v>70</v>
-      </c>
-      <c r="G28" s="32"/>
-      <c r="H28" s="24"/>
-      <c r="I28" s="28"/>
-      <c r="J28" s="24"/>
-      <c r="K28" s="28"/>
-      <c r="L28" s="28"/>
+        <v>66</v>
+      </c>
+      <c r="G28" s="30"/>
+      <c r="H28" s="22"/>
+      <c r="I28" s="23"/>
+      <c r="J28" s="22"/>
+      <c r="K28" s="23"/>
+      <c r="L28" s="23"/>
     </row>
     <row r="29" spans="1:12" ht="204" x14ac:dyDescent="0.2">
-      <c r="A29" s="23" t="s">
-        <v>71</v>
+      <c r="A29" s="2" t="s">
+        <v>67</v>
       </c>
       <c r="B29" s="2" t="s">
         <v>2</v>
       </c>
       <c r="C29" s="11" t="s">
-        <v>72</v>
+        <v>68</v>
       </c>
       <c r="D29" s="7" t="s">
-        <v>301</v>
+        <v>293</v>
       </c>
       <c r="E29" s="7" t="s">
         <v>12</v>
       </c>
       <c r="F29" s="2" t="s">
-        <v>73</v>
+        <v>69</v>
       </c>
       <c r="G29" s="5" t="s">
-        <v>314</v>
+        <v>306</v>
       </c>
       <c r="H29" s="2" t="s">
-        <v>237</v>
+        <v>230</v>
       </c>
       <c r="I29" s="2" t="s">
-        <v>74</v>
+        <v>70</v>
       </c>
       <c r="J29" s="2" t="s">
         <v>7</v>
@@ -2690,21 +2672,21 @@
         <v>31</v>
       </c>
       <c r="L29" s="2" t="s">
-        <v>298</v>
+        <v>290</v>
       </c>
     </row>
     <row r="30" spans="1:12" ht="42" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A30" s="24" t="s">
-        <v>75</v>
-      </c>
-      <c r="B30" s="25" t="s">
-        <v>55</v>
-      </c>
-      <c r="C30" s="29" t="s">
-        <v>76</v>
-      </c>
-      <c r="D30" s="30" t="s">
-        <v>77</v>
+      <c r="A30" s="22" t="s">
+        <v>71</v>
+      </c>
+      <c r="B30" s="24" t="s">
+        <v>51</v>
+      </c>
+      <c r="C30" s="27" t="s">
+        <v>72</v>
+      </c>
+      <c r="D30" s="28" t="s">
+        <v>73</v>
       </c>
       <c r="E30" s="3" t="s">
         <v>10</v>
@@ -2712,222 +2694,222 @@
       <c r="F30" s="2" t="s">
         <v>11</v>
       </c>
-      <c r="G30" s="27" t="s">
-        <v>297</v>
-      </c>
-      <c r="H30" s="25" t="s">
-        <v>246</v>
-      </c>
-      <c r="I30" s="24" t="s">
-        <v>148</v>
-      </c>
-      <c r="J30" s="24" t="s">
+      <c r="G30" s="26" t="s">
+        <v>289</v>
+      </c>
+      <c r="H30" s="24" t="s">
+        <v>239</v>
+      </c>
+      <c r="I30" s="22" t="s">
+        <v>144</v>
+      </c>
+      <c r="J30" s="22" t="s">
         <v>7</v>
       </c>
-      <c r="K30" s="24" t="s">
+      <c r="K30" s="22" t="s">
         <v>8</v>
       </c>
-      <c r="L30" s="24" t="s">
-        <v>149</v>
+      <c r="L30" s="22" t="s">
+        <v>145</v>
       </c>
     </row>
     <row r="31" spans="1:12" ht="45" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A31" s="24"/>
-      <c r="B31" s="25"/>
-      <c r="C31" s="24"/>
-      <c r="D31" s="31"/>
+      <c r="A31" s="22"/>
+      <c r="B31" s="24"/>
+      <c r="C31" s="22"/>
+      <c r="D31" s="29"/>
       <c r="E31" s="7" t="s">
         <v>12</v>
       </c>
       <c r="F31" s="2" t="s">
-        <v>78</v>
-      </c>
-      <c r="G31" s="32"/>
-      <c r="H31" s="25"/>
-      <c r="I31" s="28"/>
-      <c r="J31" s="24"/>
-      <c r="K31" s="28"/>
-      <c r="L31" s="28"/>
+        <v>74</v>
+      </c>
+      <c r="G31" s="30"/>
+      <c r="H31" s="24"/>
+      <c r="I31" s="23"/>
+      <c r="J31" s="22"/>
+      <c r="K31" s="23"/>
+      <c r="L31" s="23"/>
     </row>
     <row r="32" spans="1:12" ht="80" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A32" s="24"/>
-      <c r="B32" s="25"/>
-      <c r="C32" s="24"/>
+      <c r="A32" s="22"/>
+      <c r="B32" s="24"/>
+      <c r="C32" s="22"/>
       <c r="D32" s="3" t="s">
-        <v>79</v>
+        <v>75</v>
       </c>
       <c r="E32" s="7" t="s">
-        <v>80</v>
+        <v>76</v>
       </c>
       <c r="F32" s="2" t="s">
-        <v>81</v>
-      </c>
-      <c r="G32" s="32"/>
-      <c r="H32" s="25"/>
-      <c r="I32" s="28"/>
-      <c r="J32" s="24"/>
-      <c r="K32" s="28"/>
-      <c r="L32" s="28"/>
+        <v>77</v>
+      </c>
+      <c r="G32" s="30"/>
+      <c r="H32" s="24"/>
+      <c r="I32" s="23"/>
+      <c r="J32" s="22"/>
+      <c r="K32" s="23"/>
+      <c r="L32" s="23"/>
     </row>
     <row r="33" spans="1:12" ht="221" x14ac:dyDescent="0.2">
       <c r="A33" s="2" t="s">
+        <v>78</v>
+      </c>
+      <c r="B33" s="22" t="s">
+        <v>143</v>
+      </c>
+      <c r="C33" s="13" t="s">
+        <v>79</v>
+      </c>
+      <c r="D33" s="3" t="s">
+        <v>80</v>
+      </c>
+      <c r="E33" s="12" t="s">
+        <v>81</v>
+      </c>
+      <c r="F33" s="2" t="s">
         <v>82</v>
       </c>
-      <c r="B33" s="24" t="s">
+      <c r="G33" s="5" t="s">
+        <v>146</v>
+      </c>
+      <c r="H33" s="2" t="s">
+        <v>240</v>
+      </c>
+      <c r="I33" s="2" t="s">
+        <v>311</v>
+      </c>
+      <c r="J33" s="2" t="s">
+        <v>254</v>
+      </c>
+      <c r="K33" s="2" t="s">
+        <v>83</v>
+      </c>
+      <c r="L33" s="2" t="s">
         <v>147</v>
       </c>
-      <c r="C33" s="13" t="s">
-        <v>83</v>
-      </c>
-      <c r="D33" s="3" t="s">
+    </row>
+    <row r="34" spans="1:12" ht="68" x14ac:dyDescent="0.2">
+      <c r="A34" s="22" t="s">
         <v>84</v>
       </c>
-      <c r="E33" s="12" t="s">
+      <c r="B34" s="24"/>
+      <c r="C34" s="2" t="s">
+        <v>203</v>
+      </c>
+      <c r="D34" s="7" t="s">
+        <v>292</v>
+      </c>
+      <c r="E34" s="12" t="s">
         <v>85</v>
       </c>
-      <c r="F33" s="2" t="s">
+      <c r="F34" s="2" t="s">
+        <v>284</v>
+      </c>
+      <c r="G34" s="26" t="s">
+        <v>285</v>
+      </c>
+      <c r="H34" s="22" t="s">
+        <v>291</v>
+      </c>
+      <c r="I34" s="22" t="s">
+        <v>310</v>
+      </c>
+      <c r="J34" s="22" t="s">
+        <v>7</v>
+      </c>
+      <c r="K34" s="22" t="s">
+        <v>151</v>
+      </c>
+      <c r="L34" s="22" t="s">
+        <v>205</v>
+      </c>
+    </row>
+    <row r="35" spans="1:12" ht="51" x14ac:dyDescent="0.2">
+      <c r="A35" s="22"/>
+      <c r="B35" s="24"/>
+      <c r="C35" s="15" t="s">
         <v>86</v>
       </c>
-      <c r="G33" s="5" t="s">
-        <v>150</v>
-      </c>
-      <c r="H33" s="2" t="s">
-        <v>247</v>
-      </c>
-      <c r="I33" s="2" t="s">
-        <v>319</v>
-      </c>
-      <c r="J33" s="2" t="s">
-        <v>261</v>
-      </c>
-      <c r="K33" s="2" t="s">
+      <c r="D35" s="7" t="s">
+        <v>294</v>
+      </c>
+      <c r="E35" s="7" t="s">
         <v>87</v>
       </c>
-      <c r="L33" s="2" t="s">
-        <v>151</v>
-      </c>
-    </row>
-    <row r="34" spans="1:12" ht="68" x14ac:dyDescent="0.2">
-      <c r="A34" s="42" t="s">
+      <c r="F35" s="2" t="s">
         <v>88</v>
       </c>
-      <c r="B34" s="25"/>
-      <c r="C34" s="2" t="s">
-        <v>208</v>
-      </c>
-      <c r="D34" s="7" t="s">
-        <v>300</v>
-      </c>
-      <c r="E34" s="12" t="s">
-        <v>89</v>
-      </c>
-      <c r="F34" s="2" t="s">
-        <v>292</v>
-      </c>
-      <c r="G34" s="27" t="s">
-        <v>293</v>
-      </c>
-      <c r="H34" s="24" t="s">
-        <v>299</v>
-      </c>
-      <c r="I34" s="24" t="s">
-        <v>318</v>
-      </c>
-      <c r="J34" s="24" t="s">
-        <v>7</v>
-      </c>
-      <c r="K34" s="24" t="s">
-        <v>155</v>
-      </c>
-      <c r="L34" s="24" t="s">
-        <v>210</v>
-      </c>
-    </row>
-    <row r="35" spans="1:12" ht="51" x14ac:dyDescent="0.2">
-      <c r="A35" s="42"/>
-      <c r="B35" s="25"/>
-      <c r="C35" s="15" t="s">
-        <v>90</v>
-      </c>
-      <c r="D35" s="7" t="s">
-        <v>302</v>
-      </c>
-      <c r="E35" s="7" t="s">
-        <v>91</v>
-      </c>
-      <c r="F35" s="2" t="s">
-        <v>92</v>
-      </c>
-      <c r="G35" s="32"/>
-      <c r="H35" s="24"/>
-      <c r="I35" s="28"/>
-      <c r="J35" s="24"/>
-      <c r="K35" s="28"/>
-      <c r="L35" s="28"/>
+      <c r="G35" s="30"/>
+      <c r="H35" s="22"/>
+      <c r="I35" s="23"/>
+      <c r="J35" s="22"/>
+      <c r="K35" s="23"/>
+      <c r="L35" s="23"/>
     </row>
     <row r="36" spans="1:12" ht="221" x14ac:dyDescent="0.2">
       <c r="A36" s="2" t="s">
-        <v>152</v>
-      </c>
-      <c r="B36" s="25"/>
+        <v>148</v>
+      </c>
+      <c r="B36" s="24"/>
       <c r="C36" s="13" t="s">
+        <v>79</v>
+      </c>
+      <c r="D36" s="3" t="s">
+        <v>89</v>
+      </c>
+      <c r="E36" s="12" t="s">
+        <v>90</v>
+      </c>
+      <c r="F36" s="2" t="s">
+        <v>91</v>
+      </c>
+      <c r="G36" s="5" t="s">
+        <v>149</v>
+      </c>
+      <c r="H36" s="2" t="s">
+        <v>240</v>
+      </c>
+      <c r="I36" s="2" t="s">
+        <v>309</v>
+      </c>
+      <c r="J36" s="2" t="s">
+        <v>254</v>
+      </c>
+      <c r="K36" s="2" t="s">
         <v>83</v>
       </c>
-      <c r="D36" s="3" t="s">
-        <v>93</v>
-      </c>
-      <c r="E36" s="12" t="s">
-        <v>94</v>
-      </c>
-      <c r="F36" s="2" t="s">
-        <v>95</v>
-      </c>
-      <c r="G36" s="5" t="s">
-        <v>153</v>
-      </c>
-      <c r="H36" s="2" t="s">
-        <v>247</v>
-      </c>
-      <c r="I36" s="2" t="s">
-        <v>317</v>
-      </c>
-      <c r="J36" s="2" t="s">
-        <v>261</v>
-      </c>
-      <c r="K36" s="2" t="s">
-        <v>87</v>
-      </c>
       <c r="L36" s="2" t="s">
-        <v>154</v>
+        <v>150</v>
       </c>
     </row>
     <row r="37" spans="1:12" ht="119" x14ac:dyDescent="0.2">
       <c r="A37" s="2" t="s">
-        <v>134</v>
-      </c>
-      <c r="B37" s="25" t="s">
-        <v>55</v>
+        <v>130</v>
+      </c>
+      <c r="B37" s="24" t="s">
+        <v>51</v>
       </c>
       <c r="C37" s="4" t="s">
-        <v>213</v>
+        <v>208</v>
       </c>
       <c r="D37" s="6" t="s">
-        <v>215</v>
+        <v>210</v>
       </c>
       <c r="E37" s="9" t="s">
         <v>4</v>
       </c>
       <c r="F37" s="2" t="s">
-        <v>214</v>
+        <v>209</v>
       </c>
       <c r="G37" s="5" t="s">
-        <v>216</v>
-      </c>
-      <c r="H37" s="24" t="s">
-        <v>159</v>
-      </c>
-      <c r="I37" s="21" t="s">
-        <v>212</v>
+        <v>211</v>
+      </c>
+      <c r="H37" s="22" t="s">
+        <v>155</v>
+      </c>
+      <c r="I37" s="20" t="s">
+        <v>207</v>
       </c>
       <c r="J37" s="2" t="s">
         <v>30</v>
@@ -2936,160 +2918,160 @@
         <v>31</v>
       </c>
       <c r="L37" s="2" t="s">
-        <v>268</v>
+        <v>261</v>
       </c>
     </row>
     <row r="38" spans="1:12" ht="187" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A38" s="24" t="s">
-        <v>160</v>
-      </c>
-      <c r="B38" s="25"/>
-      <c r="C38" s="41" t="s">
-        <v>217</v>
-      </c>
-      <c r="D38" s="40" t="s">
-        <v>219</v>
+      <c r="A38" s="22" t="s">
+        <v>156</v>
+      </c>
+      <c r="B38" s="24"/>
+      <c r="C38" s="37" t="s">
+        <v>212</v>
+      </c>
+      <c r="D38" s="36" t="s">
+        <v>214</v>
       </c>
       <c r="E38" s="3" t="s">
         <v>10</v>
       </c>
       <c r="F38" s="2" t="s">
-        <v>223</v>
-      </c>
-      <c r="G38" s="27" t="s">
-        <v>224</v>
-      </c>
-      <c r="H38" s="24"/>
-      <c r="I38" s="25" t="s">
-        <v>212</v>
-      </c>
-      <c r="J38" s="24" t="s">
+        <v>218</v>
+      </c>
+      <c r="G38" s="26" t="s">
+        <v>219</v>
+      </c>
+      <c r="H38" s="22"/>
+      <c r="I38" s="24" t="s">
+        <v>207</v>
+      </c>
+      <c r="J38" s="22" t="s">
         <v>30</v>
       </c>
-      <c r="K38" s="24" t="s">
+      <c r="K38" s="22" t="s">
         <v>31</v>
       </c>
-      <c r="L38" s="25" t="s">
-        <v>268</v>
+      <c r="L38" s="24" t="s">
+        <v>261</v>
       </c>
     </row>
     <row r="39" spans="1:12" ht="17" x14ac:dyDescent="0.2">
-      <c r="A39" s="24"/>
-      <c r="B39" s="25"/>
-      <c r="C39" s="41"/>
-      <c r="D39" s="40"/>
+      <c r="A39" s="22"/>
+      <c r="B39" s="24"/>
+      <c r="C39" s="37"/>
+      <c r="D39" s="36"/>
       <c r="E39" s="4" t="s">
-        <v>101</v>
+        <v>97</v>
       </c>
       <c r="F39" s="2" t="s">
-        <v>222</v>
-      </c>
-      <c r="G39" s="27"/>
-      <c r="H39" s="24"/>
-      <c r="I39" s="25"/>
-      <c r="J39" s="24"/>
-      <c r="K39" s="24"/>
-      <c r="L39" s="25"/>
+        <v>217</v>
+      </c>
+      <c r="G39" s="26"/>
+      <c r="H39" s="22"/>
+      <c r="I39" s="24"/>
+      <c r="J39" s="22"/>
+      <c r="K39" s="22"/>
+      <c r="L39" s="24"/>
     </row>
     <row r="40" spans="1:12" ht="34" x14ac:dyDescent="0.2">
-      <c r="A40" s="24"/>
-      <c r="B40" s="25"/>
-      <c r="C40" s="41"/>
+      <c r="A40" s="22"/>
+      <c r="B40" s="24"/>
+      <c r="C40" s="37"/>
       <c r="D40" s="3" t="s">
-        <v>218</v>
+        <v>213</v>
       </c>
       <c r="E40" s="7" t="s">
         <v>12</v>
       </c>
       <c r="F40" s="2" t="s">
-        <v>221</v>
-      </c>
-      <c r="G40" s="27"/>
-      <c r="H40" s="24"/>
-      <c r="I40" s="25"/>
-      <c r="J40" s="24"/>
-      <c r="K40" s="24"/>
-      <c r="L40" s="25"/>
+        <v>216</v>
+      </c>
+      <c r="G40" s="26"/>
+      <c r="H40" s="22"/>
+      <c r="I40" s="24"/>
+      <c r="J40" s="22"/>
+      <c r="K40" s="22"/>
+      <c r="L40" s="24"/>
     </row>
     <row r="41" spans="1:12" ht="77" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A41" s="34" t="s">
-        <v>96</v>
-      </c>
-      <c r="B41" s="24" t="s">
-        <v>97</v>
-      </c>
-      <c r="C41" s="39" t="s">
-        <v>98</v>
-      </c>
-      <c r="D41" s="40" t="s">
-        <v>99</v>
+      <c r="A41" s="31" t="s">
+        <v>92</v>
+      </c>
+      <c r="B41" s="22" t="s">
+        <v>93</v>
+      </c>
+      <c r="C41" s="35" t="s">
+        <v>94</v>
+      </c>
+      <c r="D41" s="36" t="s">
+        <v>95</v>
       </c>
       <c r="E41" s="3" t="s">
         <v>10</v>
       </c>
       <c r="F41" s="2" t="s">
+        <v>96</v>
+      </c>
+      <c r="G41" s="26" t="s">
+        <v>160</v>
+      </c>
+      <c r="H41" s="22" t="s">
+        <v>152</v>
+      </c>
+      <c r="I41" s="22" t="s">
+        <v>157</v>
+      </c>
+      <c r="J41" s="22" t="s">
+        <v>30</v>
+      </c>
+      <c r="K41" s="22" t="s">
+        <v>31</v>
+      </c>
+      <c r="L41" s="22" t="s">
+        <v>159</v>
+      </c>
+    </row>
+    <row r="42" spans="1:12" ht="73" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A42" s="22"/>
+      <c r="B42" s="22"/>
+      <c r="C42" s="22"/>
+      <c r="D42" s="33"/>
+      <c r="E42" s="4" t="s">
+        <v>97</v>
+      </c>
+      <c r="F42" s="2" t="s">
+        <v>215</v>
+      </c>
+      <c r="G42" s="30"/>
+      <c r="H42" s="22"/>
+      <c r="I42" s="23"/>
+      <c r="J42" s="22"/>
+      <c r="K42" s="23"/>
+      <c r="L42" s="23"/>
+    </row>
+    <row r="43" spans="1:12" ht="272" x14ac:dyDescent="0.2">
+      <c r="A43" s="21" t="s">
+        <v>99</v>
+      </c>
+      <c r="B43" s="22"/>
+      <c r="C43" s="16" t="s">
         <v>100</v>
       </c>
-      <c r="G41" s="27" t="s">
-        <v>164</v>
-      </c>
-      <c r="H41" s="24" t="s">
-        <v>156</v>
-      </c>
-      <c r="I41" s="24" t="s">
-        <v>161</v>
-      </c>
-      <c r="J41" s="24" t="s">
-        <v>30</v>
-      </c>
-      <c r="K41" s="24" t="s">
-        <v>31</v>
-      </c>
-      <c r="L41" s="24" t="s">
-        <v>163</v>
-      </c>
-    </row>
-    <row r="42" spans="1:12" ht="73" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A42" s="24"/>
-      <c r="B42" s="24"/>
-      <c r="C42" s="24"/>
-      <c r="D42" s="36"/>
-      <c r="E42" s="4" t="s">
+      <c r="D43" s="3" t="s">
         <v>101</v>
       </c>
-      <c r="F42" s="2" t="s">
-        <v>220</v>
-      </c>
-      <c r="G42" s="32"/>
-      <c r="H42" s="24"/>
-      <c r="I42" s="28"/>
-      <c r="J42" s="24"/>
-      <c r="K42" s="28"/>
-      <c r="L42" s="28"/>
-    </row>
-    <row r="43" spans="1:12" ht="272" x14ac:dyDescent="0.2">
-      <c r="A43" s="16" t="s">
-        <v>103</v>
-      </c>
-      <c r="B43" s="24"/>
-      <c r="C43" s="17" t="s">
-        <v>104</v>
-      </c>
-      <c r="D43" s="3" t="s">
-        <v>105</v>
-      </c>
       <c r="E43" s="4" t="s">
-        <v>101</v>
+        <v>97</v>
       </c>
       <c r="F43" s="2" t="s">
-        <v>220</v>
+        <v>215</v>
       </c>
       <c r="G43" s="5" t="s">
-        <v>166</v>
-      </c>
-      <c r="H43" s="24"/>
+        <v>162</v>
+      </c>
+      <c r="H43" s="22"/>
       <c r="I43" s="2" t="s">
-        <v>161</v>
+        <v>157</v>
       </c>
       <c r="J43" s="2" t="s">
         <v>30</v>
@@ -3098,32 +3080,32 @@
         <v>31</v>
       </c>
       <c r="L43" s="2" t="s">
-        <v>165</v>
+        <v>161</v>
       </c>
     </row>
     <row r="44" spans="1:12" ht="255" x14ac:dyDescent="0.2">
-      <c r="A44" s="16" t="s">
-        <v>106</v>
-      </c>
-      <c r="B44" s="24"/>
-      <c r="C44" s="17" t="s">
-        <v>107</v>
+      <c r="A44" s="21" t="s">
+        <v>102</v>
+      </c>
+      <c r="B44" s="22"/>
+      <c r="C44" s="16" t="s">
+        <v>103</v>
       </c>
       <c r="D44" s="3" t="s">
-        <v>108</v>
+        <v>104</v>
       </c>
       <c r="E44" s="4" t="s">
-        <v>101</v>
+        <v>97</v>
       </c>
       <c r="F44" s="2" t="s">
-        <v>102</v>
+        <v>98</v>
       </c>
       <c r="G44" s="5" t="s">
-        <v>167</v>
-      </c>
-      <c r="H44" s="24"/>
+        <v>163</v>
+      </c>
+      <c r="H44" s="22"/>
       <c r="I44" s="2" t="s">
-        <v>161</v>
+        <v>157</v>
       </c>
       <c r="J44" s="2" t="s">
         <v>30</v>
@@ -3132,159 +3114,159 @@
         <v>31</v>
       </c>
       <c r="L44" s="2" t="s">
-        <v>168</v>
+        <v>164</v>
       </c>
     </row>
     <row r="45" spans="1:12" ht="112" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A45" s="34" t="s">
-        <v>109</v>
-      </c>
-      <c r="B45" s="24"/>
-      <c r="C45" s="39" t="s">
-        <v>109</v>
-      </c>
-      <c r="D45" s="40" t="s">
-        <v>110</v>
+      <c r="A45" s="31" t="s">
+        <v>105</v>
+      </c>
+      <c r="B45" s="22"/>
+      <c r="C45" s="35" t="s">
+        <v>105</v>
+      </c>
+      <c r="D45" s="36" t="s">
+        <v>106</v>
       </c>
       <c r="E45" s="3" t="s">
         <v>10</v>
       </c>
       <c r="F45" s="2" t="s">
-        <v>100</v>
-      </c>
-      <c r="G45" s="27" t="s">
-        <v>170</v>
-      </c>
-      <c r="H45" s="24"/>
-      <c r="I45" s="24" t="s">
-        <v>169</v>
-      </c>
-      <c r="J45" s="24" t="s">
+        <v>96</v>
+      </c>
+      <c r="G45" s="26" t="s">
+        <v>166</v>
+      </c>
+      <c r="H45" s="22"/>
+      <c r="I45" s="22" t="s">
+        <v>165</v>
+      </c>
+      <c r="J45" s="22" t="s">
         <v>30</v>
       </c>
-      <c r="K45" s="24" t="s">
+      <c r="K45" s="22" t="s">
         <v>31</v>
       </c>
-      <c r="L45" s="24" t="s">
-        <v>171</v>
+      <c r="L45" s="22" t="s">
+        <v>167</v>
       </c>
     </row>
     <row r="46" spans="1:12" ht="98" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A46" s="24"/>
-      <c r="B46" s="24"/>
-      <c r="C46" s="24"/>
-      <c r="D46" s="36"/>
+      <c r="A46" s="22"/>
+      <c r="B46" s="22"/>
+      <c r="C46" s="22"/>
+      <c r="D46" s="33"/>
       <c r="E46" s="3" t="s">
-        <v>101</v>
+        <v>97</v>
       </c>
       <c r="F46" s="2" t="s">
-        <v>111</v>
-      </c>
-      <c r="G46" s="32"/>
-      <c r="H46" s="24"/>
-      <c r="I46" s="28"/>
-      <c r="J46" s="24"/>
-      <c r="K46" s="28"/>
-      <c r="L46" s="28"/>
+        <v>107</v>
+      </c>
+      <c r="G46" s="30"/>
+      <c r="H46" s="22"/>
+      <c r="I46" s="23"/>
+      <c r="J46" s="22"/>
+      <c r="K46" s="23"/>
+      <c r="L46" s="23"/>
     </row>
     <row r="47" spans="1:12" ht="84" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A47" s="34" t="s">
-        <v>123</v>
-      </c>
-      <c r="B47" s="24"/>
-      <c r="C47" s="39" t="s">
-        <v>124</v>
+      <c r="A47" s="31" t="s">
+        <v>119</v>
+      </c>
+      <c r="B47" s="22"/>
+      <c r="C47" s="35" t="s">
+        <v>120</v>
       </c>
       <c r="D47" s="7" t="s">
-        <v>125</v>
+        <v>121</v>
       </c>
       <c r="E47" s="7" t="s">
         <v>12</v>
       </c>
       <c r="F47" s="2" t="s">
-        <v>126</v>
-      </c>
-      <c r="G47" s="27" t="s">
-        <v>157</v>
-      </c>
-      <c r="H47" s="24"/>
-      <c r="I47" s="24" t="s">
-        <v>162</v>
-      </c>
-      <c r="J47" s="24" t="s">
+        <v>122</v>
+      </c>
+      <c r="G47" s="26" t="s">
+        <v>153</v>
+      </c>
+      <c r="H47" s="22"/>
+      <c r="I47" s="22" t="s">
+        <v>158</v>
+      </c>
+      <c r="J47" s="22" t="s">
         <v>30</v>
       </c>
-      <c r="K47" s="24" t="s">
+      <c r="K47" s="22" t="s">
         <v>31</v>
       </c>
-      <c r="L47" s="24" t="s">
-        <v>158</v>
+      <c r="L47" s="22" t="s">
+        <v>154</v>
       </c>
     </row>
     <row r="48" spans="1:12" ht="47" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A48" s="24"/>
-      <c r="B48" s="24"/>
-      <c r="C48" s="24"/>
+      <c r="A48" s="22"/>
+      <c r="B48" s="22"/>
+      <c r="C48" s="22"/>
       <c r="D48" s="3" t="s">
-        <v>127</v>
+        <v>123</v>
       </c>
       <c r="E48" s="4" t="s">
-        <v>101</v>
+        <v>97</v>
       </c>
       <c r="F48" s="2" t="s">
-        <v>111</v>
-      </c>
-      <c r="G48" s="32"/>
-      <c r="H48" s="24"/>
-      <c r="I48" s="28"/>
-      <c r="J48" s="24"/>
-      <c r="K48" s="28"/>
-      <c r="L48" s="28"/>
+        <v>107</v>
+      </c>
+      <c r="G48" s="30"/>
+      <c r="H48" s="22"/>
+      <c r="I48" s="23"/>
+      <c r="J48" s="22"/>
+      <c r="K48" s="23"/>
+      <c r="L48" s="23"/>
     </row>
     <row r="49" spans="1:12" ht="104" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A49" s="34" t="s">
-        <v>112</v>
-      </c>
-      <c r="B49" s="24"/>
-      <c r="C49" s="19" t="s">
-        <v>113</v>
+      <c r="A49" s="31" t="s">
+        <v>108</v>
+      </c>
+      <c r="B49" s="22"/>
+      <c r="C49" s="18" t="s">
+        <v>109</v>
       </c>
       <c r="D49" s="6" t="s">
-        <v>175</v>
+        <v>171</v>
       </c>
       <c r="E49" s="3" t="s">
         <v>10</v>
       </c>
       <c r="F49" s="2" t="s">
-        <v>114</v>
-      </c>
-      <c r="G49" s="27" t="s">
-        <v>177</v>
-      </c>
-      <c r="H49" s="24" t="s">
-        <v>172</v>
-      </c>
-      <c r="I49" s="24" t="s">
+        <v>110</v>
+      </c>
+      <c r="G49" s="26" t="s">
         <v>173</v>
       </c>
-      <c r="J49" s="24" t="s">
+      <c r="H49" s="22" t="s">
+        <v>168</v>
+      </c>
+      <c r="I49" s="22" t="s">
+        <v>169</v>
+      </c>
+      <c r="J49" s="22" t="s">
         <v>30</v>
       </c>
-      <c r="K49" s="24" t="s">
+      <c r="K49" s="22" t="s">
         <v>31</v>
       </c>
-      <c r="L49" s="24" t="s">
-        <v>163</v>
+      <c r="L49" s="22" t="s">
+        <v>159</v>
       </c>
     </row>
     <row r="50" spans="1:12" ht="62" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A50" s="24"/>
-      <c r="B50" s="24"/>
+      <c r="A50" s="22"/>
+      <c r="B50" s="22"/>
       <c r="C50" s="11" t="s">
-        <v>226</v>
+        <v>221</v>
       </c>
       <c r="D50" s="7" t="s">
-        <v>53</v>
+        <v>49</v>
       </c>
       <c r="E50" s="7" t="s">
         <v>12</v>
@@ -3292,125 +3274,125 @@
       <c r="F50" s="2" t="s">
         <v>33</v>
       </c>
-      <c r="G50" s="32"/>
-      <c r="H50" s="24"/>
-      <c r="I50" s="28"/>
-      <c r="J50" s="24"/>
-      <c r="K50" s="28"/>
-      <c r="L50" s="28"/>
+      <c r="G50" s="30"/>
+      <c r="H50" s="22"/>
+      <c r="I50" s="23"/>
+      <c r="J50" s="22"/>
+      <c r="K50" s="23"/>
+      <c r="L50" s="23"/>
     </row>
     <row r="51" spans="1:12" ht="113" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A51" s="34" t="s">
-        <v>115</v>
-      </c>
-      <c r="B51" s="24"/>
-      <c r="C51" s="35" t="s">
-        <v>116</v>
+      <c r="A51" s="31" t="s">
+        <v>111</v>
+      </c>
+      <c r="B51" s="22"/>
+      <c r="C51" s="32" t="s">
+        <v>112</v>
       </c>
       <c r="D51" s="6" t="s">
-        <v>176</v>
+        <v>172</v>
       </c>
       <c r="E51" s="3" t="s">
         <v>10</v>
       </c>
       <c r="F51" s="2" t="s">
-        <v>111</v>
-      </c>
-      <c r="G51" s="27" t="s">
-        <v>308</v>
-      </c>
-      <c r="H51" s="24"/>
-      <c r="I51" s="24" t="s">
-        <v>179</v>
-      </c>
-      <c r="J51" s="24" t="s">
+        <v>107</v>
+      </c>
+      <c r="G51" s="26" t="s">
+        <v>300</v>
+      </c>
+      <c r="H51" s="22"/>
+      <c r="I51" s="22" t="s">
+        <v>175</v>
+      </c>
+      <c r="J51" s="22" t="s">
         <v>7</v>
       </c>
-      <c r="K51" s="24" t="s">
+      <c r="K51" s="22" t="s">
         <v>31</v>
       </c>
-      <c r="L51" s="24" t="s">
-        <v>178</v>
+      <c r="L51" s="22" t="s">
+        <v>174</v>
       </c>
     </row>
     <row r="52" spans="1:12" ht="50" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A52" s="34"/>
-      <c r="B52" s="24"/>
-      <c r="C52" s="24"/>
-      <c r="D52" s="31" t="s">
-        <v>53</v>
-      </c>
-      <c r="E52" s="31" t="s">
+      <c r="A52" s="31"/>
+      <c r="B52" s="22"/>
+      <c r="C52" s="22"/>
+      <c r="D52" s="29" t="s">
+        <v>49</v>
+      </c>
+      <c r="E52" s="29" t="s">
         <v>12</v>
       </c>
       <c r="F52" s="2" t="s">
-        <v>117</v>
-      </c>
-      <c r="G52" s="27"/>
-      <c r="H52" s="24"/>
-      <c r="I52" s="24"/>
-      <c r="J52" s="24"/>
-      <c r="K52" s="24"/>
-      <c r="L52" s="24"/>
+        <v>113</v>
+      </c>
+      <c r="G52" s="26"/>
+      <c r="H52" s="22"/>
+      <c r="I52" s="22"/>
+      <c r="J52" s="22"/>
+      <c r="K52" s="22"/>
+      <c r="L52" s="22"/>
     </row>
     <row r="53" spans="1:12" ht="17" x14ac:dyDescent="0.2">
-      <c r="A53" s="34"/>
-      <c r="B53" s="24"/>
+      <c r="A53" s="31"/>
+      <c r="B53" s="22"/>
       <c r="C53" s="11" t="s">
-        <v>226</v>
-      </c>
-      <c r="D53" s="31"/>
-      <c r="E53" s="31"/>
+        <v>221</v>
+      </c>
+      <c r="D53" s="29"/>
+      <c r="E53" s="29"/>
       <c r="F53" s="2" t="s">
         <v>33</v>
       </c>
-      <c r="G53" s="27"/>
-      <c r="H53" s="24"/>
-      <c r="I53" s="24"/>
-      <c r="J53" s="24"/>
-      <c r="K53" s="24"/>
-      <c r="L53" s="24"/>
+      <c r="G53" s="26"/>
+      <c r="H53" s="22"/>
+      <c r="I53" s="22"/>
+      <c r="J53" s="22"/>
+      <c r="K53" s="22"/>
+      <c r="L53" s="22"/>
     </row>
     <row r="54" spans="1:12" ht="187" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A54" s="34" t="s">
-        <v>118</v>
-      </c>
-      <c r="B54" s="24"/>
-      <c r="C54" s="33" t="s">
-        <v>315</v>
+      <c r="A54" s="31" t="s">
+        <v>114</v>
+      </c>
+      <c r="B54" s="22"/>
+      <c r="C54" s="34" t="s">
+        <v>307</v>
       </c>
       <c r="D54" s="3" t="s">
-        <v>119</v>
+        <v>115</v>
       </c>
       <c r="E54" s="4" t="s">
         <v>4</v>
       </c>
       <c r="F54" s="2" t="s">
-        <v>120</v>
-      </c>
-      <c r="G54" s="27" t="s">
-        <v>196</v>
-      </c>
-      <c r="H54" s="24"/>
-      <c r="I54" s="24" t="s">
-        <v>181</v>
-      </c>
-      <c r="J54" s="24" t="s">
+        <v>116</v>
+      </c>
+      <c r="G54" s="26" t="s">
+        <v>192</v>
+      </c>
+      <c r="H54" s="22"/>
+      <c r="I54" s="22" t="s">
+        <v>177</v>
+      </c>
+      <c r="J54" s="22" t="s">
         <v>30</v>
       </c>
-      <c r="K54" s="24" t="s">
+      <c r="K54" s="22" t="s">
         <v>31</v>
       </c>
-      <c r="L54" s="24" t="s">
-        <v>180</v>
+      <c r="L54" s="22" t="s">
+        <v>176</v>
       </c>
     </row>
     <row r="55" spans="1:12" ht="17" x14ac:dyDescent="0.2">
-      <c r="A55" s="34"/>
-      <c r="B55" s="24"/>
-      <c r="C55" s="33"/>
+      <c r="A55" s="31"/>
+      <c r="B55" s="22"/>
+      <c r="C55" s="34"/>
       <c r="D55" s="7" t="s">
-        <v>53</v>
+        <v>49</v>
       </c>
       <c r="E55" s="7" t="s">
         <v>12</v>
@@ -3418,243 +3400,243 @@
       <c r="F55" s="2" t="s">
         <v>33</v>
       </c>
-      <c r="G55" s="27"/>
-      <c r="H55" s="24"/>
-      <c r="I55" s="24"/>
-      <c r="J55" s="24"/>
-      <c r="K55" s="24"/>
-      <c r="L55" s="24"/>
+      <c r="G55" s="26"/>
+      <c r="H55" s="22"/>
+      <c r="I55" s="22"/>
+      <c r="J55" s="22"/>
+      <c r="K55" s="22"/>
+      <c r="L55" s="22"/>
     </row>
     <row r="56" spans="1:12" ht="94" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A56" s="34" t="s">
-        <v>187</v>
-      </c>
-      <c r="B56" s="24"/>
-      <c r="C56" s="33" t="s">
-        <v>206</v>
+      <c r="A56" s="31" t="s">
+        <v>183</v>
+      </c>
+      <c r="B56" s="22"/>
+      <c r="C56" s="34" t="s">
+        <v>201</v>
       </c>
       <c r="D56" s="8" t="s">
-        <v>202</v>
+        <v>198</v>
       </c>
       <c r="E56" s="7" t="s">
         <v>12</v>
       </c>
       <c r="F56" s="2" t="s">
-        <v>192</v>
-      </c>
-      <c r="G56" s="27" t="s">
+        <v>188</v>
+      </c>
+      <c r="G56" s="26" t="s">
+        <v>182</v>
+      </c>
+      <c r="H56" s="22"/>
+      <c r="I56" s="22" t="s">
+        <v>181</v>
+      </c>
+      <c r="J56" s="22" t="s">
+        <v>30</v>
+      </c>
+      <c r="K56" s="22" t="s">
+        <v>31</v>
+      </c>
+      <c r="L56" s="22" t="s">
+        <v>180</v>
+      </c>
+    </row>
+    <row r="57" spans="1:12" ht="80" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A57" s="22"/>
+      <c r="B57" s="22"/>
+      <c r="C57" s="22"/>
+      <c r="D57" s="3" t="s">
+        <v>178</v>
+      </c>
+      <c r="E57" s="4" t="s">
+        <v>97</v>
+      </c>
+      <c r="F57" s="2" t="s">
+        <v>179</v>
+      </c>
+      <c r="G57" s="30"/>
+      <c r="H57" s="22"/>
+      <c r="I57" s="23"/>
+      <c r="J57" s="22"/>
+      <c r="K57" s="23"/>
+      <c r="L57" s="23"/>
+    </row>
+    <row r="58" spans="1:12" ht="107" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A58" s="31" t="s">
+        <v>184</v>
+      </c>
+      <c r="B58" s="22" t="s">
+        <v>143</v>
+      </c>
+      <c r="C58" s="34" t="s">
+        <v>202</v>
+      </c>
+      <c r="D58" s="3" t="s">
         <v>186</v>
-      </c>
-      <c r="H56" s="24"/>
-      <c r="I56" s="24" t="s">
-        <v>185</v>
-      </c>
-      <c r="J56" s="24" t="s">
-        <v>30</v>
-      </c>
-      <c r="K56" s="24" t="s">
-        <v>31</v>
-      </c>
-      <c r="L56" s="24" t="s">
-        <v>184</v>
-      </c>
-    </row>
-    <row r="57" spans="1:12" ht="80" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A57" s="24"/>
-      <c r="B57" s="24"/>
-      <c r="C57" s="24"/>
-      <c r="D57" s="3" t="s">
-        <v>182</v>
-      </c>
-      <c r="E57" s="4" t="s">
-        <v>101</v>
-      </c>
-      <c r="F57" s="2" t="s">
-        <v>183</v>
-      </c>
-      <c r="G57" s="32"/>
-      <c r="H57" s="24"/>
-      <c r="I57" s="28"/>
-      <c r="J57" s="24"/>
-      <c r="K57" s="28"/>
-      <c r="L57" s="28"/>
-    </row>
-    <row r="58" spans="1:12" ht="107" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A58" s="34" t="s">
-        <v>188</v>
-      </c>
-      <c r="B58" s="24" t="s">
-        <v>147</v>
-      </c>
-      <c r="C58" s="33" t="s">
-        <v>207</v>
-      </c>
-      <c r="D58" s="3" t="s">
-        <v>190</v>
       </c>
       <c r="E58" s="4" t="s">
         <v>4</v>
       </c>
       <c r="F58" s="2" t="s">
-        <v>193</v>
-      </c>
-      <c r="G58" s="27" t="s">
-        <v>195</v>
-      </c>
-      <c r="H58" s="24"/>
-      <c r="I58" s="24" t="s">
-        <v>194</v>
-      </c>
-      <c r="J58" s="24" t="s">
+        <v>189</v>
+      </c>
+      <c r="G58" s="26" t="s">
+        <v>191</v>
+      </c>
+      <c r="H58" s="22"/>
+      <c r="I58" s="22" t="s">
+        <v>190</v>
+      </c>
+      <c r="J58" s="22" t="s">
         <v>30</v>
       </c>
-      <c r="K58" s="24" t="s">
+      <c r="K58" s="22" t="s">
         <v>31</v>
       </c>
-      <c r="L58" s="24" t="s">
-        <v>189</v>
+      <c r="L58" s="22" t="s">
+        <v>185</v>
       </c>
     </row>
     <row r="59" spans="1:12" ht="72" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A59" s="24"/>
-      <c r="B59" s="24"/>
-      <c r="C59" s="24"/>
+      <c r="A59" s="22"/>
+      <c r="B59" s="22"/>
+      <c r="C59" s="22"/>
       <c r="D59" s="7" t="s">
-        <v>53</v>
+        <v>49</v>
       </c>
       <c r="E59" s="7" t="s">
         <v>12</v>
       </c>
       <c r="F59" s="2" t="s">
-        <v>191</v>
-      </c>
-      <c r="G59" s="32"/>
-      <c r="H59" s="24"/>
-      <c r="I59" s="28"/>
-      <c r="J59" s="24"/>
-      <c r="K59" s="28"/>
-      <c r="L59" s="28"/>
+        <v>187</v>
+      </c>
+      <c r="G59" s="30"/>
+      <c r="H59" s="22"/>
+      <c r="I59" s="23"/>
+      <c r="J59" s="22"/>
+      <c r="K59" s="23"/>
+      <c r="L59" s="23"/>
     </row>
     <row r="60" spans="1:12" ht="34" x14ac:dyDescent="0.2">
-      <c r="A60" s="34" t="s">
-        <v>199</v>
-      </c>
-      <c r="B60" s="24" t="s">
-        <v>97</v>
-      </c>
-      <c r="C60" s="33" t="s">
-        <v>200</v>
+      <c r="A60" s="31" t="s">
+        <v>195</v>
+      </c>
+      <c r="B60" s="22" t="s">
+        <v>93</v>
+      </c>
+      <c r="C60" s="34" t="s">
+        <v>196</v>
       </c>
       <c r="D60" s="7" t="s">
-        <v>121</v>
+        <v>117</v>
       </c>
       <c r="E60" s="7" t="s">
         <v>12</v>
       </c>
       <c r="F60" s="2" t="s">
-        <v>191</v>
-      </c>
-      <c r="G60" s="27" t="s">
-        <v>204</v>
-      </c>
-      <c r="H60" s="24" t="s">
-        <v>246</v>
-      </c>
-      <c r="I60" s="24" t="s">
-        <v>205</v>
-      </c>
-      <c r="J60" s="24" t="s">
-        <v>261</v>
-      </c>
-      <c r="K60" s="24" t="s">
+        <v>187</v>
+      </c>
+      <c r="G60" s="26" t="s">
+        <v>322</v>
+      </c>
+      <c r="H60" s="22" t="s">
+        <v>239</v>
+      </c>
+      <c r="I60" s="22" t="s">
+        <v>200</v>
+      </c>
+      <c r="J60" s="22" t="s">
+        <v>254</v>
+      </c>
+      <c r="K60" s="22" t="s">
         <v>8</v>
       </c>
-      <c r="L60" s="24" t="s">
-        <v>270</v>
+      <c r="L60" s="22" t="s">
+        <v>263</v>
       </c>
     </row>
     <row r="61" spans="1:12" ht="68" x14ac:dyDescent="0.2">
-      <c r="A61" s="24"/>
-      <c r="B61" s="24"/>
-      <c r="C61" s="24"/>
+      <c r="A61" s="22"/>
+      <c r="B61" s="22"/>
+      <c r="C61" s="22"/>
       <c r="D61" s="7" t="s">
-        <v>203</v>
+        <v>199</v>
       </c>
       <c r="E61" s="4" t="s">
-        <v>122</v>
+        <v>118</v>
       </c>
       <c r="F61" s="2" t="s">
-        <v>201</v>
-      </c>
-      <c r="G61" s="32"/>
-      <c r="H61" s="24"/>
-      <c r="I61" s="28"/>
-      <c r="J61" s="24"/>
-      <c r="K61" s="28"/>
-      <c r="L61" s="28"/>
+        <v>197</v>
+      </c>
+      <c r="G61" s="30"/>
+      <c r="H61" s="22"/>
+      <c r="I61" s="23"/>
+      <c r="J61" s="22"/>
+      <c r="K61" s="23"/>
+      <c r="L61" s="23"/>
     </row>
     <row r="62" spans="1:12" ht="83" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A62" s="34" t="s">
-        <v>271</v>
-      </c>
-      <c r="B62" s="24" t="s">
-        <v>97</v>
-      </c>
-      <c r="C62" s="35" t="s">
+      <c r="A62" s="31" t="s">
+        <v>264</v>
+      </c>
+      <c r="B62" s="22" t="s">
+        <v>93</v>
+      </c>
+      <c r="C62" s="32" t="s">
+        <v>124</v>
+      </c>
+      <c r="D62" s="6" t="s">
+        <v>125</v>
+      </c>
+      <c r="E62" s="33" t="s">
+        <v>10</v>
+      </c>
+      <c r="F62" s="2" t="s">
+        <v>126</v>
+      </c>
+      <c r="G62" s="26" t="s">
+        <v>265</v>
+      </c>
+      <c r="H62" s="22" t="s">
+        <v>239</v>
+      </c>
+      <c r="I62" s="22" t="s">
+        <v>127</v>
+      </c>
+      <c r="J62" s="22" t="s">
+        <v>7</v>
+      </c>
+      <c r="K62" s="22" t="s">
+        <v>8</v>
+      </c>
+      <c r="L62" s="22" t="s">
         <v>128</v>
       </c>
-      <c r="D62" s="6" t="s">
+    </row>
+    <row r="63" spans="1:12" ht="90" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A63" s="31"/>
+      <c r="B63" s="22"/>
+      <c r="C63" s="32"/>
+      <c r="D63" s="6" t="s">
+        <v>55</v>
+      </c>
+      <c r="E63" s="33"/>
+      <c r="F63" s="2" t="s">
         <v>129</v>
       </c>
-      <c r="E62" s="36" t="s">
-        <v>10</v>
-      </c>
-      <c r="F62" s="2" t="s">
-        <v>130</v>
-      </c>
-      <c r="G62" s="27" t="s">
-        <v>272</v>
-      </c>
-      <c r="H62" s="24" t="s">
-        <v>246</v>
-      </c>
-      <c r="I62" s="37" t="s">
-        <v>131</v>
-      </c>
-      <c r="J62" s="24" t="s">
-        <v>7</v>
-      </c>
-      <c r="K62" s="24" t="s">
-        <v>8</v>
-      </c>
-      <c r="L62" s="24" t="s">
-        <v>132</v>
-      </c>
-    </row>
-    <row r="63" spans="1:12" ht="90" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A63" s="34"/>
-      <c r="B63" s="24"/>
-      <c r="C63" s="35"/>
-      <c r="D63" s="6" t="s">
-        <v>59</v>
-      </c>
-      <c r="E63" s="36"/>
-      <c r="F63" s="2" t="s">
-        <v>133</v>
-      </c>
-      <c r="G63" s="27"/>
-      <c r="H63" s="24"/>
-      <c r="I63" s="37"/>
-      <c r="J63" s="24"/>
-      <c r="K63" s="24"/>
-      <c r="L63" s="24"/>
+      <c r="G63" s="26"/>
+      <c r="H63" s="22"/>
+      <c r="I63" s="22"/>
+      <c r="J63" s="22"/>
+      <c r="K63" s="22"/>
+      <c r="L63" s="22"/>
     </row>
     <row r="64" spans="1:12" ht="64" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A64" s="24"/>
-      <c r="B64" s="24"/>
-      <c r="C64" s="24"/>
+      <c r="A64" s="22"/>
+      <c r="B64" s="22"/>
+      <c r="C64" s="22"/>
       <c r="D64" s="7" t="s">
-        <v>53</v>
+        <v>49</v>
       </c>
       <c r="E64" s="7" t="s">
         <v>12</v>
@@ -3662,12 +3644,12 @@
       <c r="F64" s="2" t="s">
         <v>33</v>
       </c>
-      <c r="G64" s="32"/>
-      <c r="H64" s="24"/>
-      <c r="I64" s="38"/>
-      <c r="J64" s="24"/>
-      <c r="K64" s="28"/>
-      <c r="L64" s="28"/>
+      <c r="G64" s="30"/>
+      <c r="H64" s="22"/>
+      <c r="I64" s="23"/>
+      <c r="J64" s="22"/>
+      <c r="K64" s="23"/>
+      <c r="L64" s="23"/>
     </row>
   </sheetData>
   <mergeCells count="192">
@@ -3727,6 +3709,7 @@
     <mergeCell ref="A12:A13"/>
     <mergeCell ref="G12:G13"/>
     <mergeCell ref="I12:I13"/>
+    <mergeCell ref="J12:J13"/>
     <mergeCell ref="A17:A19"/>
     <mergeCell ref="B17:B19"/>
     <mergeCell ref="C17:C19"/>
@@ -3736,7 +3719,6 @@
     <mergeCell ref="B24:B26"/>
     <mergeCell ref="G24:G26"/>
     <mergeCell ref="H24:H26"/>
-    <mergeCell ref="J12:J13"/>
     <mergeCell ref="C24:C25"/>
     <mergeCell ref="L17:L19"/>
     <mergeCell ref="G17:G19"/>
@@ -3747,6 +3729,7 @@
     <mergeCell ref="D21:D22"/>
     <mergeCell ref="I24:I26"/>
     <mergeCell ref="I30:I32"/>
+    <mergeCell ref="K27:K28"/>
     <mergeCell ref="A27:A28"/>
     <mergeCell ref="B27:B28"/>
     <mergeCell ref="C27:C28"/>
@@ -3758,6 +3741,7 @@
     <mergeCell ref="A34:A35"/>
     <mergeCell ref="G34:G35"/>
     <mergeCell ref="I34:I35"/>
+    <mergeCell ref="J27:J28"/>
     <mergeCell ref="K34:K35"/>
     <mergeCell ref="G38:G40"/>
     <mergeCell ref="A38:A40"/>
@@ -3769,7 +3753,7 @@
     <mergeCell ref="J38:J40"/>
     <mergeCell ref="K38:K40"/>
     <mergeCell ref="H34:H35"/>
-    <mergeCell ref="J27:J28"/>
+    <mergeCell ref="J34:J35"/>
     <mergeCell ref="I56:I57"/>
     <mergeCell ref="K56:K57"/>
     <mergeCell ref="L56:L57"/>
@@ -3792,7 +3776,6 @@
     <mergeCell ref="H41:H48"/>
     <mergeCell ref="J45:J46"/>
     <mergeCell ref="J41:J42"/>
-    <mergeCell ref="K27:K28"/>
     <mergeCell ref="J49:J50"/>
     <mergeCell ref="A51:A53"/>
     <mergeCell ref="J58:J59"/>
@@ -3862,7 +3845,6 @@
     <mergeCell ref="C30:C32"/>
     <mergeCell ref="D30:D31"/>
     <mergeCell ref="G30:G32"/>
-    <mergeCell ref="J34:J35"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" horizontalDpi="0" verticalDpi="0"/>
@@ -3879,189 +3861,189 @@
   <sheetData>
     <row r="1" spans="1:11" s="1" customFormat="1" ht="115" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A1" s="1" t="s">
-        <v>274</v>
+        <v>267</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>262</v>
+        <v>255</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>275</v>
+        <v>268</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>276</v>
+        <v>269</v>
       </c>
       <c r="E1" s="1" t="s">
-        <v>277</v>
+        <v>270</v>
       </c>
       <c r="F1" s="1" t="s">
-        <v>278</v>
+        <v>271</v>
       </c>
       <c r="G1" s="1" t="s">
-        <v>263</v>
+        <v>256</v>
       </c>
       <c r="H1" s="1" t="s">
-        <v>279</v>
+        <v>316</v>
       </c>
       <c r="I1" s="1" t="s">
-        <v>260</v>
+        <v>253</v>
       </c>
       <c r="J1" s="1" t="s">
-        <v>265</v>
+        <v>258</v>
       </c>
       <c r="K1" s="2" t="s">
-        <v>174</v>
+        <v>170</v>
       </c>
     </row>
     <row r="2" spans="1:11" ht="115" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B2" s="2" t="s">
-        <v>243</v>
+        <v>236</v>
       </c>
       <c r="C2" s="4" t="s">
-        <v>135</v>
+        <v>131</v>
       </c>
       <c r="D2" s="4" t="s">
-        <v>136</v>
+        <v>132</v>
       </c>
       <c r="E2" s="4" t="s">
-        <v>316</v>
+        <v>308</v>
       </c>
       <c r="F2" s="4"/>
       <c r="G2" s="2" t="s">
-        <v>250</v>
+        <v>243</v>
       </c>
       <c r="I2" s="2" t="s">
-        <v>256</v>
-      </c>
-      <c r="J2" s="20" t="s">
-        <v>269</v>
+        <v>249</v>
+      </c>
+      <c r="J2" s="19" t="s">
+        <v>262</v>
       </c>
     </row>
     <row r="3" spans="1:11" ht="115" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B3" s="2" t="s">
-        <v>244</v>
+        <v>237</v>
       </c>
       <c r="C3" s="8" t="s">
-        <v>137</v>
+        <v>133</v>
       </c>
       <c r="D3" s="8" t="s">
-        <v>138</v>
+        <v>134</v>
       </c>
       <c r="E3" s="8" t="s">
         <v>14</v>
       </c>
       <c r="F3" s="8"/>
       <c r="G3" s="2" t="s">
-        <v>254</v>
+        <v>247</v>
       </c>
       <c r="I3" s="2" t="s">
-        <v>257</v>
-      </c>
-      <c r="J3" s="20" t="s">
-        <v>313</v>
+        <v>250</v>
+      </c>
+      <c r="J3" s="19" t="s">
+        <v>305</v>
       </c>
     </row>
     <row r="4" spans="1:11" ht="115" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B4" s="2" t="s">
-        <v>242</v>
+        <v>235</v>
       </c>
       <c r="C4" s="3" t="s">
-        <v>139</v>
+        <v>135</v>
       </c>
       <c r="D4" s="3" t="s">
-        <v>140</v>
+        <v>136</v>
       </c>
       <c r="E4" s="3" t="s">
         <v>10</v>
       </c>
       <c r="F4" s="3"/>
       <c r="G4" s="2" t="s">
-        <v>253</v>
+        <v>246</v>
       </c>
       <c r="I4" s="2" t="s">
-        <v>258</v>
-      </c>
-      <c r="J4" s="20" t="s">
-        <v>249</v>
+        <v>251</v>
+      </c>
+      <c r="J4" s="19" t="s">
+        <v>242</v>
       </c>
     </row>
     <row r="5" spans="1:11" ht="115" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B5" s="2" t="s">
-        <v>252</v>
+        <v>245</v>
       </c>
       <c r="C5" s="7" t="s">
-        <v>141</v>
+        <v>137</v>
       </c>
       <c r="D5" s="7" t="s">
-        <v>142</v>
+        <v>138</v>
       </c>
       <c r="E5" s="7" t="s">
         <v>12</v>
       </c>
       <c r="F5" s="7"/>
       <c r="G5" s="2" t="s">
-        <v>251</v>
-      </c>
-      <c r="J5" s="20" t="s">
-        <v>211</v>
+        <v>244</v>
+      </c>
+      <c r="J5" s="19" t="s">
+        <v>206</v>
       </c>
     </row>
     <row r="6" spans="1:11" ht="115" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B6" s="2" t="s">
-        <v>295</v>
+        <v>287</v>
       </c>
       <c r="C6" s="12" t="s">
-        <v>143</v>
-      </c>
-      <c r="D6" s="18" t="s">
-        <v>264</v>
+        <v>139</v>
+      </c>
+      <c r="D6" s="17" t="s">
+        <v>257</v>
       </c>
       <c r="E6" s="12" t="s">
-        <v>89</v>
+        <v>85</v>
       </c>
       <c r="F6" s="12"/>
       <c r="G6" s="2" t="s">
-        <v>197</v>
+        <v>193</v>
       </c>
     </row>
     <row r="7" spans="1:11" ht="115" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B7" s="2" t="s">
-        <v>305</v>
+        <v>297</v>
       </c>
       <c r="C7" s="13" t="s">
-        <v>83</v>
+        <v>79</v>
       </c>
       <c r="E7" s="13" t="s">
-        <v>144</v>
+        <v>140</v>
       </c>
       <c r="F7" s="13"/>
       <c r="G7" s="2" t="s">
-        <v>198</v>
+        <v>194</v>
       </c>
     </row>
     <row r="8" spans="1:11" ht="115" customHeight="1" x14ac:dyDescent="0.2">
       <c r="C8" s="15" t="s">
-        <v>145</v>
+        <v>141</v>
       </c>
       <c r="G8" s="2" t="s">
-        <v>255</v>
+        <v>248</v>
       </c>
     </row>
     <row r="9" spans="1:11" ht="115" customHeight="1" x14ac:dyDescent="0.2">
       <c r="C9" s="14" t="s">
-        <v>146</v>
+        <v>142</v>
       </c>
     </row>
     <row r="10" spans="1:11" ht="115" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="J10" s="20"/>
+      <c r="J10" s="19"/>
     </row>
     <row r="11" spans="1:11" ht="115" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="J11" s="20"/>
+      <c r="J11" s="19"/>
     </row>
     <row r="13" spans="1:11" ht="115" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="J13" s="20"/>
+      <c r="J13" s="19"/>
     </row>
     <row r="14" spans="1:11" ht="115" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="J14" s="20"/>
+      <c r="J14" s="19"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>